<commit_message>
feat(comercial): fecha funil de captacao e alinha site com CRM
- Centraliza configuracao do WhatsApp em site-config.js
- Impede envio quando numero esta em placeholder
- Alinha formulario com CRM e modelo de turmas
- Adiciona campo de dificuldade
- Inclui origem do lead na mensagem WhatsApp
- Remove links internos do footer publico
- Adiciona aviso de privacidade
- Adiciona validacoes required
- Atualiza README para arquitetura v0.6

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/operacional/CRM-Template.xlsx
+++ b/operacional/CRM-Template.xlsx
@@ -746,12 +746,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>6o ano</t>
+          <t>6º ano fundamental</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Matematica</t>
+          <t>Matemática</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -786,9 +786,15 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="5">
     <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Escolha um status da lista padronizada." prompt="Status do funil comercial" type="list">
       <formula1>"🟡 Interessado,🔵 Contato realizado,🟠 Visita agendada,🟣 Avaliacao realizada,🟢 Matricula realizada,🔴 Nao interessado,⚫ Lista de espera"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"4º ano fundamental,5º ano fundamental,6º ano fundamental,7º ano fundamental,8º ano fundamental,9º ano fundamental,1º ano ensino médio,2º ano ensino médio,3º ano ensino médio,Reforço para provas"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Matemática,Português / leitura,Ciências,Organização e estudos,Múltiplas disciplinas,Outro"</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Manha,Tarde,Noite"</formula1>

</xml_diff>